<commit_message>
implemented tau to deg conversion
to do: build wrapper around Servo
</commit_message>
<xml_diff>
--- a/notes/Weight Budget.xlsx
+++ b/notes/Weight Budget.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alexc\Documents\GitHub\leonidas-lander\notes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E48FEC3-77E7-481D-B60C-66A605D9687A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47E97421-9221-4BF4-AAC2-F06CEC4E2169}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{F5F24785-2A24-44CD-ABA3-ADA57A5DC66F}"/>
+    <workbookView xWindow="-105" yWindow="10440" windowWidth="19410" windowHeight="10545" xr2:uid="{F5F24785-2A24-44CD-ABA3-ADA57A5DC66F}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="45">
   <si>
     <t>Item</t>
   </si>
@@ -138,6 +138,42 @@
   </si>
   <si>
     <t>estimated</t>
+  </si>
+  <si>
+    <t>Turnigy Nano-Tech Plus 3000mAh 3S 70C LiPo Battery Pack w/XT90</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>Turnigy Heavy Duty 5000mAh 3S 60C Lipo Pack w/XT-90</t>
+  </si>
+  <si>
+    <t>Weight</t>
+  </si>
+  <si>
+    <t>Ah</t>
+  </si>
+  <si>
+    <t>Turnigy Heavy Duty 5000mAh 6S 60C LiPo Pack avec XT90</t>
+  </si>
+  <si>
+    <t>S</t>
+  </si>
+  <si>
+    <t>S*kg/Ah</t>
+  </si>
+  <si>
+    <t>W</t>
+  </si>
+  <si>
+    <t>kgf</t>
+  </si>
+  <si>
+    <t>V</t>
+  </si>
+  <si>
+    <t>A</t>
   </si>
 </sst>
 </file>
@@ -312,7 +348,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -375,6 +411,7 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
@@ -1699,16 +1736,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>162358</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>10824</xdr:rowOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>757417</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>55873</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>36</xdr:col>
-      <xdr:colOff>100263</xdr:colOff>
-      <xdr:row>59</xdr:row>
-      <xdr:rowOff>26831</xdr:rowOff>
+      <xdr:col>39</xdr:col>
+      <xdr:colOff>695323</xdr:colOff>
+      <xdr:row>71</xdr:row>
+      <xdr:rowOff>71881</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2053,16 +2090,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C7F43134-4BEF-4687-9116-4D9336CD4254}">
-  <dimension ref="A1:P34"/>
+  <dimension ref="A1:Z34"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.140625" customWidth="1"/>
     <col min="2" max="2" width="12.7109375" customWidth="1"/>
     <col min="5" max="5" width="3.140625" customWidth="1"/>
     <col min="15" max="15" width="11.42578125" customWidth="1"/>
+    <col min="21" max="21" width="82.42578125" customWidth="1"/>
+    <col min="24" max="25" width="11.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A1" s="27" t="s">
         <v>20</v>
       </c>
@@ -2073,7 +2112,7 @@
       <c r="F1" s="27"/>
       <c r="G1" s="27"/>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A2" s="27"/>
       <c r="B2" s="27"/>
       <c r="C2" s="27"/>
@@ -2082,7 +2121,7 @@
       <c r="F2" s="27"/>
       <c r="G2" s="27"/>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>0</v>
       </c>
@@ -2096,8 +2135,26 @@
         <v>3</v>
       </c>
       <c r="E3" s="29"/>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="U3" t="s">
+        <v>0</v>
+      </c>
+      <c r="V3" t="s">
+        <v>34</v>
+      </c>
+      <c r="W3" t="s">
+        <v>36</v>
+      </c>
+      <c r="X3" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>39</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
         <v>4</v>
       </c>
@@ -2131,8 +2188,27 @@
       <c r="P4" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="U4" s="30" t="s">
+        <v>33</v>
+      </c>
+      <c r="V4">
+        <v>4</v>
+      </c>
+      <c r="W4">
+        <v>287</v>
+      </c>
+      <c r="X4">
+        <v>3</v>
+      </c>
+      <c r="Y4">
+        <v>3</v>
+      </c>
+      <c r="Z4">
+        <f>W4/1000/X4/Y4</f>
+        <v>3.188888888888889E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
         <v>6</v>
       </c>
@@ -2166,8 +2242,27 @@
       <c r="P5" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="U5" s="30" t="s">
+        <v>35</v>
+      </c>
+      <c r="V5">
+        <v>4</v>
+      </c>
+      <c r="W5">
+        <v>440</v>
+      </c>
+      <c r="X5">
+        <v>6</v>
+      </c>
+      <c r="Y5">
+        <v>3</v>
+      </c>
+      <c r="Z5">
+        <f t="shared" ref="Z5:Z6" si="1">W5/1000/X5/Y5</f>
+        <v>2.4444444444444446E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A6" s="15" t="s">
         <v>29</v>
       </c>
@@ -2202,8 +2297,27 @@
       <c r="P6" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="U6" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="V6">
+        <v>2</v>
+      </c>
+      <c r="W6">
+        <v>838</v>
+      </c>
+      <c r="X6">
+        <v>5</v>
+      </c>
+      <c r="Y6">
+        <v>6</v>
+      </c>
+      <c r="Z6">
+        <f t="shared" si="1"/>
+        <v>2.7933333333333334E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A7" s="13" t="s">
         <v>9</v>
       </c>
@@ -2221,7 +2335,7 @@
       <c r="I7" s="1"/>
       <c r="J7" s="1"/>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
         <v>10</v>
       </c>
@@ -2250,7 +2364,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
         <v>25</v>
       </c>
@@ -2269,7 +2383,7 @@
       </c>
       <c r="F9" s="4"/>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
         <v>21</v>
       </c>
@@ -2287,8 +2401,14 @@
         <v>5</v>
       </c>
       <c r="F10" s="4"/>
-    </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="O10">
+        <v>304.3</v>
+      </c>
+      <c r="Q10">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
         <v>22</v>
       </c>
@@ -2307,7 +2427,7 @@
       </c>
       <c r="F11" s="4"/>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
         <v>23</v>
       </c>
@@ -2323,8 +2443,20 @@
       </c>
       <c r="E12" s="7"/>
       <c r="F12" s="4"/>
-    </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="O12" t="s">
+        <v>42</v>
+      </c>
+      <c r="P12" t="s">
+        <v>41</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>43</v>
+      </c>
+      <c r="R12" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="13" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
         <v>24</v>
       </c>
@@ -2342,8 +2474,23 @@
         <v>5</v>
       </c>
       <c r="F13" s="4"/>
-    </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="O13">
+        <v>0.1</v>
+      </c>
+      <c r="P13">
+        <f>O$10*(O13^(3/2))</f>
+        <v>9.6228109198923804</v>
+      </c>
+      <c r="Q13">
+        <f>Q$10*4.2</f>
+        <v>25.200000000000003</v>
+      </c>
+      <c r="R13">
+        <f>P13/Q13</f>
+        <v>0.38185757618620553</v>
+      </c>
+    </row>
+    <row r="14" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A14" s="13" t="s">
         <v>12</v>
       </c>
@@ -2362,8 +2509,23 @@
         <v>5</v>
       </c>
       <c r="F14" s="4"/>
-    </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="O14">
+        <v>0.25</v>
+      </c>
+      <c r="P14">
+        <f t="shared" ref="P14:P21" si="2">O$10*(O14^(3/2))</f>
+        <v>38.037500000000009</v>
+      </c>
+      <c r="Q14">
+        <f t="shared" ref="Q14:Q21" si="3">Q$10*4.2</f>
+        <v>25.200000000000003</v>
+      </c>
+      <c r="R14">
+        <f t="shared" ref="R14:R21" si="4">P14/Q14</f>
+        <v>1.5094246031746033</v>
+      </c>
+    </row>
+    <row r="15" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A15" s="23" t="s">
         <v>31</v>
       </c>
@@ -2381,8 +2543,24 @@
         <v>5</v>
       </c>
       <c r="F15" s="4"/>
-    </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="O15">
+        <f>O14*2</f>
+        <v>0.5</v>
+      </c>
+      <c r="P15">
+        <f t="shared" si="2"/>
+        <v>107.58629675753322</v>
+      </c>
+      <c r="Q15">
+        <f t="shared" si="3"/>
+        <v>25.200000000000003</v>
+      </c>
+      <c r="R15">
+        <f t="shared" si="4"/>
+        <v>4.2692974903783023</v>
+      </c>
+    </row>
+    <row r="16" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A16" s="19" t="s">
         <v>13</v>
       </c>
@@ -2400,8 +2578,24 @@
         <v>5</v>
       </c>
       <c r="F16" s="4"/>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="O16">
+        <f>O15*2</f>
+        <v>1</v>
+      </c>
+      <c r="P16">
+        <f t="shared" si="2"/>
+        <v>304.3</v>
+      </c>
+      <c r="Q16">
+        <f t="shared" si="3"/>
+        <v>25.200000000000003</v>
+      </c>
+      <c r="R16">
+        <f t="shared" si="4"/>
+        <v>12.075396825396824</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A17" s="19" t="s">
         <v>14</v>
       </c>
@@ -2419,8 +2613,24 @@
         <v>5</v>
       </c>
       <c r="F17" s="4"/>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="O17">
+        <f>O16*2</f>
+        <v>2</v>
+      </c>
+      <c r="P17">
+        <f t="shared" si="2"/>
+        <v>860.69037406026564</v>
+      </c>
+      <c r="Q17">
+        <f t="shared" si="3"/>
+        <v>25.200000000000003</v>
+      </c>
+      <c r="R17">
+        <f t="shared" si="4"/>
+        <v>34.154379923026411</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A18" s="14" t="s">
         <v>15</v>
       </c>
@@ -2438,8 +2648,23 @@
         <v>5</v>
       </c>
       <c r="F18" s="4"/>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="O18">
+        <v>2.5</v>
+      </c>
+      <c r="P18">
+        <f t="shared" si="2"/>
+        <v>1202.8513649865474</v>
+      </c>
+      <c r="Q18">
+        <f t="shared" si="3"/>
+        <v>25.200000000000003</v>
+      </c>
+      <c r="R18">
+        <f t="shared" si="4"/>
+        <v>47.732197023275688</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
         <v>16</v>
       </c>
@@ -2457,8 +2682,23 @@
         <v>5</v>
       </c>
       <c r="F19" s="4"/>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="O19">
+        <v>3</v>
+      </c>
+      <c r="P19">
+        <f t="shared" si="2"/>
+        <v>1581.1891822296282</v>
+      </c>
+      <c r="Q19">
+        <f t="shared" si="3"/>
+        <v>25.200000000000003</v>
+      </c>
+      <c r="R19">
+        <f t="shared" si="4"/>
+        <v>62.745602469429684</v>
+      </c>
+    </row>
+    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
         <v>17</v>
       </c>
@@ -2474,8 +2714,23 @@
         <v>5</v>
       </c>
       <c r="F20" s="4"/>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="O20">
+        <v>3.5</v>
+      </c>
+      <c r="P20">
+        <f t="shared" si="2"/>
+        <v>1992.5260998917936</v>
+      </c>
+      <c r="Q20">
+        <f t="shared" si="3"/>
+        <v>25.200000000000003</v>
+      </c>
+      <c r="R20">
+        <f t="shared" si="4"/>
+        <v>79.068496027452113</v>
+      </c>
+    </row>
+    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A21" s="13" t="s">
         <v>18</v>
       </c>
@@ -2491,8 +2746,23 @@
         <v>5</v>
       </c>
       <c r="F21" s="4"/>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="O21">
+        <v>3.8</v>
+      </c>
+      <c r="P21">
+        <f t="shared" si="2"/>
+        <v>2254.1216345352796</v>
+      </c>
+      <c r="Q21">
+        <f t="shared" si="3"/>
+        <v>25.200000000000003</v>
+      </c>
+      <c r="R21">
+        <f t="shared" si="4"/>
+        <v>89.449271211717431</v>
+      </c>
+    </row>
+    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A22" s="23" t="s">
         <v>19</v>
       </c>
@@ -2511,7 +2781,7 @@
       </c>
       <c r="F22" s="4"/>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A23" s="18" t="s">
         <v>30</v>
       </c>
@@ -2530,7 +2800,7 @@
       </c>
       <c r="F23" s="4"/>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A24" s="13"/>
       <c r="B24" s="22"/>
       <c r="C24" s="1"/>
@@ -2543,7 +2813,7 @@
       </c>
       <c r="F24" s="4"/>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A25" s="13"/>
       <c r="B25" s="22"/>
       <c r="C25" s="1"/>
@@ -2551,7 +2821,7 @@
       <c r="E25" s="1"/>
       <c r="F25" s="4"/>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A26" s="13"/>
       <c r="B26" s="22"/>
       <c r="C26" s="1"/>
@@ -2559,7 +2829,7 @@
       <c r="E26" s="1"/>
       <c r="F26" s="4"/>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A27" s="13"/>
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
@@ -2567,7 +2837,7 @@
       <c r="E27" s="1"/>
       <c r="F27" s="4"/>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A28" s="13"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
@@ -2575,7 +2845,7 @@
       <c r="E28" s="1"/>
       <c r="F28" s="4"/>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A29" s="13"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
@@ -2583,7 +2853,7 @@
       <c r="E29" s="1"/>
       <c r="F29" s="4"/>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A30" s="13"/>
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
@@ -2591,7 +2861,7 @@
       <c r="E30" s="1"/>
       <c r="F30" s="4"/>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A31" s="13"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
@@ -2599,7 +2869,7 @@
       <c r="E31" s="1"/>
       <c r="F31" s="4"/>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A32" s="13"/>
       <c r="B32" s="1"/>
       <c r="C32" s="1"/>
@@ -2633,8 +2903,11 @@
     <hyperlink ref="A8" r:id="rId2" xr:uid="{6CFE664B-910F-4B72-BAD9-44B28ABF7916}"/>
     <hyperlink ref="A6" r:id="rId3" xr:uid="{39CF0902-36CF-48A1-A2B5-4D86A9F166A5}"/>
     <hyperlink ref="A23" r:id="rId4" xr:uid="{9B054A69-B1E8-4635-BDA3-D7F9B30F1DAA}"/>
+    <hyperlink ref="U4" r:id="rId5" location="search/BATTERY/FMfcgzQXJQTdcZjlcFhLGxLmQZFnshJL" xr:uid="{AE2053A0-3FED-40FE-AF6D-289F7A4ECA02}"/>
+    <hyperlink ref="U5" r:id="rId6" location="search/BATTERY/FMfcgzGrbvHZNWMMMMXtbdGVsKSvQLzm" xr:uid="{A7A44006-5A76-42A9-B2FC-10C440BE6441}"/>
+    <hyperlink ref="U6" r:id="rId7" xr:uid="{912B8DC0-0A64-47FB-B6F1-49912AA1BEAC}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId5"/>
+  <drawing r:id="rId8"/>
 </worksheet>
 </file>
</xml_diff>